<commit_message>
read data from the excel file
</commit_message>
<xml_diff>
--- a/src/test/java/testData/TestData.xlsx
+++ b/src/test/java/testData/TestData.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a83364ae384c52e2/Documents/2026/Ndosi Automation/Selenium Java/Group5AdvancedFormAutomation/src/test/java/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{39DBBDFE-5393-4865-81F9-EA2CF5BDC524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D673B2E3-DB81-486B-9B30-4FB8A2789AB0}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{39DBBDFE-5393-4865-81F9-EA2CF5BDC524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BDE170D-9C2E-402F-96AC-E2236E54865A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Information Tab" sheetId="2" r:id="rId1"/>
     <sheet name="Login Details" sheetId="1" r:id="rId2"/>
+    <sheet name="Inventory Details" sheetId="3" r:id="rId3"/>
+    <sheet name="Extras Details" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>Username</t>
   </si>
@@ -76,6 +78,57 @@
   </si>
   <si>
     <t>@123456789</t>
+  </si>
+  <si>
+    <t>DeviceType</t>
+  </si>
+  <si>
+    <t>Brand</t>
+  </si>
+  <si>
+    <t>Storage</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>128GB</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>123 Test Address</t>
+  </si>
+  <si>
+    <t>Shipping Method</t>
+  </si>
+  <si>
+    <t>Warranty</t>
+  </si>
+  <si>
+    <t>Discount Code</t>
+  </si>
+  <si>
+    <t>Express</t>
+  </si>
+  <si>
+    <t>1 Year</t>
+  </si>
+  <si>
+    <t>SAVE10</t>
   </si>
 </sst>
 </file>
@@ -518,4 +571,99 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAD721FD-F788-4AB3-BED0-5A368ABDE061}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.7265625" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.08984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1585EB51-F423-4E17-8C17-6FE461BAD07E}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>